<commit_message>
Update pricing model with actual channel fees and September results
Direct sales carry a 7% system charge; Klook 20% and Travelers Road 17%
commission plus a 3% system charge. OTA prices now keep the same take
as direct sales. Hanko has no tour cost and stays at a flat price.
Adds a September by-channel sheet (aggregates only, no personal data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7xJuJLT164ew2d7KNvQh3
</commit_message>
<xml_diff>
--- a/docs/pricing/NGT_価格モデル.xlsx
+++ b/docs/pricing/NGT_価格モデル.xlsx
@@ -11,6 +11,7 @@
     <sheet name="公式価格（段階制）" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OTA価格" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="現行価格の収支" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="9月実績（チャネル別）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0%;(0.0%);-"/>
     <numFmt numFmtId="166" formatCode="0&quot;名&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +66,9 @@
     <font>
       <name val="Arial"/>
       <color rgb="00008000"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -116,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +144,14 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -703,11 +715,11 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>公式直販の決済・システム手数料率</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>0.05</v>
+          <t>公式直販のシステム利用料率</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
@@ -716,7 +728,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>LINKTIVITY直販エンジン＋カード決済の合計想定（推測・要確認）</t>
+          <t>実数：LINKTIVITY取引明細（2026/9）。総額に対して7%（決済込み）</t>
         </is>
       </c>
     </row>
@@ -790,12 +802,35 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ハンコツアーの催行コスト（ガイド費・材料費）</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>円/回</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ご本人確認 2026-10-02：費用はかからない</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>チャネル別の手数料</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>OTA手数料率</t>
-        </is>
-      </c>
+      <c r="A21" s="4" t="n"/>
       <c r="B21" s="5" t="n"/>
       <c r="C21" s="5" t="n"/>
       <c r="D21" s="5" t="n"/>
@@ -846,7 +881,7 @@
           <t>Klook</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="10" t="n">
         <v>0.2</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -856,7 +891,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>業界一般値の仮置き（推測）。LINKTIVITY経由の実際の契約料率に差し替え</t>
+          <t>実数：LINKTIVITY取引明細（2026/9）</t>
         </is>
       </c>
     </row>
@@ -906,8 +941,8 @@
           <t>Travelers Road（卸）</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
-        <v>0.2</v>
+      <c r="B27" s="10" t="n">
+        <v>0.17</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
@@ -916,7 +951,47 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>業界一般値の仮置き（推測）。LINKTIVITY経由の実際の契約料率に差し替え</t>
+          <t>実数：LINKTIVITY取引明細（2026/9）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Private Group</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>率</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>実数：LINKTIVITY取引明細（2026/9）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>OTA経由のシステム利用料率</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>率</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>実数：LINKTIVITY取引明細（2026/9）。OTA手数料とは別に総額の3%。キャンセル時に戻る条件は要確認</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1662,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>・12歳以下：「大人1名につき子ども1名まで無料」を推奨。ガイド費の人数区分は子どもも数えるため、無制限に無料だと大人2名＋子ども5名などで赤字になる。</t>
+          <t>・12歳以下：何人でも無料（大人の同伴が必要、2026-09-25確定）。子どもがガイド費の人数区分に数えられる場合は、その分だけ利益が下振れする。</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1676,7 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>・ハンコ代・スイーツ代などツアー固有の材料費は含まない。該当ツアーは1名あたり価格に材料費を加算する。</t>
+          <t>・ハンコ代・スイーツ代などツアー固有の材料費は含まない。ハンコツアーは費用がかからないため段階制の対象外（「OTA価格」シートの一律行）。</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1639,7 +1714,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>計算式：OTA価格 ＝ 公式価格 ÷（1 − OTA手数料率）を100円単位で切り上げ。OTA経由でも手取りが公式と同等以上になる。</t>
+          <t>計算式：OTA価格 ＝ 公式価格 ×（1 − 公式直販のシステム利用料率）÷（1 − OTA手数料率 − OTA経由のシステム利用料率）を100円単位で切り上げ。どのチャネルで売れても手取りが公式と同じになる（2026-10-02 実数で改定）。</t>
         </is>
       </c>
     </row>
@@ -1696,27 +1771,27 @@
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$22),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$22-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$23),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$23-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$24),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$24-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="F5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$25),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$25-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="G5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$26),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$26-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="H5" s="13">
-        <f>ROUNDUP($B5/(1-前提条件!$B$27),-2)</f>
+        <f>ROUNDUP($B5*(1-前提条件!$B$14)/(1-前提条件!$B$27-前提条件!$B$29),-2)</f>
         <v/>
       </c>
     </row>
@@ -1731,27 +1806,27 @@
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$22),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$22-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$23),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$23-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="E6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$24),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$24-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="F6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$25),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$25-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="G6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$26),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$26-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="H6" s="13">
-        <f>ROUNDUP($B6/(1-前提条件!$B$27),-2)</f>
+        <f>ROUNDUP($B6*(1-前提条件!$B$14)/(1-前提条件!$B$27-前提条件!$B$29),-2)</f>
         <v/>
       </c>
     </row>
@@ -1766,27 +1841,27 @@
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$22),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$22-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$23),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$23-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$24),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$24-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="F7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$25),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$25-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="G7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$26),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$26-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="H7" s="13">
-        <f>ROUNDUP($B7/(1-前提条件!$B$27),-2)</f>
+        <f>ROUNDUP($B7*(1-前提条件!$B$14)/(1-前提条件!$B$27-前提条件!$B$29),-2)</f>
         <v/>
       </c>
     </row>
@@ -1801,28 +1876,56 @@
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$22),-2)</f>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$22-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$23),-2)</f>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$23-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="E8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$24),-2)</f>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$24-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="F8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$25),-2)</f>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$25-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="G8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$26),-2)</f>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$26-前提条件!$B$29),-2)</f>
         <v/>
       </c>
       <c r="H8" s="13">
-        <f>ROUNDUP($B8/(1-前提条件!$B$27),-2)</f>
-        <v/>
+        <f>ROUNDUP($B8*(1-前提条件!$B$14)/(1-前提条件!$B$27-前提条件!$B$29),-2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ハンコ（一律）</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>3000</v>
       </c>
     </row>
     <row r="10">
@@ -1843,6 +1946,13 @@
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>・Travelers Road（卸）は卸値契約のため、上乗せではなく卸値（ネット価格）で合意する形になる可能性が高い（要確認）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>・ハンコは費用がかからないため人数に関わらず一律（青字＝入力値）。OTAは売れている¥3,000を維持（Klookの式の値¥3,100との差は1名15円）。</t>
         </is>
       </c>
     </row>
@@ -2225,4 +2335,584 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>2026年9月の実績（購入日 9/1〜9/30）：チャネル×人数別の手取りと利益、新価格での試算</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>出典：LINKTIVITY 予約一覧・取引明細（集計値のみ。個人情報は含めない）。テスト予約1件・旅行者キャンセル3件は除外。1予約＝1催行と仮定。新価格の列は同じ予約が同じ件数入った場合の試算（推測）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>チャネル</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>ツアー</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>人数（大人）</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>予約数</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>現行単価</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>OTA手数料率</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>システム利用料率</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>手取り率</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>現行の手取り</t>
+        </is>
+      </c>
+      <c r="J4" s="22" t="inlineStr">
+        <is>
+          <t>催行コスト</t>
+        </is>
+      </c>
+      <c r="K4" s="22" t="inlineStr">
+        <is>
+          <t>現行の利益</t>
+        </is>
+      </c>
+      <c r="L4" s="22" t="inlineStr">
+        <is>
+          <t>新単価</t>
+        </is>
+      </c>
+      <c r="M4" s="22" t="inlineStr">
+        <is>
+          <t>新価格の手取り</t>
+        </is>
+      </c>
+      <c r="N4" s="22" t="inlineStr">
+        <is>
+          <t>新価格の利益</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Klook</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ハンコ</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F5" s="24">
+        <f>前提条件!$B$24</f>
+        <v/>
+      </c>
+      <c r="G5" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>1-F5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="23">
+        <f>E5*C5*D5*H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="23">
+        <f>前提条件!$B$19*D5</f>
+        <v/>
+      </c>
+      <c r="K5" s="23">
+        <f>I5-J5</f>
+        <v/>
+      </c>
+      <c r="L5" s="23">
+        <f>'OTA価格'!$E$9</f>
+        <v/>
+      </c>
+      <c r="M5" s="23">
+        <f>L5*C5*D5*H5</f>
+        <v/>
+      </c>
+      <c r="N5" s="23">
+        <f>M5-J5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Klook</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ハンコ</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F6" s="24">
+        <f>前提条件!$B$24</f>
+        <v/>
+      </c>
+      <c r="G6" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>1-F6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="23">
+        <f>E6*C6*D6*H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="23">
+        <f>前提条件!$B$19*D6</f>
+        <v/>
+      </c>
+      <c r="K6" s="23">
+        <f>I6-J6</f>
+        <v/>
+      </c>
+      <c r="L6" s="23">
+        <f>'OTA価格'!$E$9</f>
+        <v/>
+      </c>
+      <c r="M6" s="23">
+        <f>L6*C6*D6*H6</f>
+        <v/>
+      </c>
+      <c r="N6" s="23">
+        <f>M6-J6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Klook</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ハンコ</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F7" s="24">
+        <f>前提条件!$B$24</f>
+        <v/>
+      </c>
+      <c r="G7" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>1-F7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="23">
+        <f>E7*C7*D7*H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="23">
+        <f>前提条件!$B$19*D7</f>
+        <v/>
+      </c>
+      <c r="K7" s="23">
+        <f>I7-J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="23">
+        <f>'OTA価格'!$E$9</f>
+        <v/>
+      </c>
+      <c r="M7" s="23">
+        <f>L7*C7*D7*H7</f>
+        <v/>
+      </c>
+      <c r="N7" s="23">
+        <f>M7-J7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Travelers Road</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>秘境神社</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F8" s="24">
+        <f>前提条件!$B$27</f>
+        <v/>
+      </c>
+      <c r="G8" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>1-F8-G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="23">
+        <f>E8*C8*D8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="23">
+        <f>(IF(C8&lt;=3,前提条件!$B$6,IF(C8&lt;=6,前提条件!$B$7,前提条件!$B$8))+前提条件!$B$13)*D8</f>
+        <v/>
+      </c>
+      <c r="K8" s="23">
+        <f>I8-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="23">
+        <f>INDEX('OTA価格'!$H$5:$H$8,MIN(C8,4))</f>
+        <v/>
+      </c>
+      <c r="M8" s="23">
+        <f>L8*C8*D8*H8</f>
+        <v/>
+      </c>
+      <c r="N8" s="23">
+        <f>M8-J8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Travelers Road</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>秘境神社</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F9" s="24">
+        <f>前提条件!$B$27</f>
+        <v/>
+      </c>
+      <c r="G9" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>1-F9-G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="23">
+        <f>E9*C9*D9*H9</f>
+        <v/>
+      </c>
+      <c r="J9" s="23">
+        <f>(IF(C9&lt;=3,前提条件!$B$6,IF(C9&lt;=6,前提条件!$B$7,前提条件!$B$8))+前提条件!$B$13)*D9</f>
+        <v/>
+      </c>
+      <c r="K9" s="23">
+        <f>I9-J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="23">
+        <f>INDEX('OTA価格'!$H$5:$H$8,MIN(C9,4))</f>
+        <v/>
+      </c>
+      <c r="M9" s="23">
+        <f>L9*C9*D9*H9</f>
+        <v/>
+      </c>
+      <c r="N9" s="23">
+        <f>M9-J9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Travelers Road</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>秘境神社</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F10" s="24">
+        <f>前提条件!$B$27</f>
+        <v/>
+      </c>
+      <c r="G10" s="24">
+        <f>前提条件!$B$29</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>1-F10-G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="23">
+        <f>E10*C10*D10*H10</f>
+        <v/>
+      </c>
+      <c r="J10" s="23">
+        <f>(IF(C10&lt;=3,前提条件!$B$6,IF(C10&lt;=6,前提条件!$B$7,前提条件!$B$8))+前提条件!$B$13)*D10</f>
+        <v/>
+      </c>
+      <c r="K10" s="23">
+        <f>I10-J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="23">
+        <f>INDEX('OTA価格'!$H$5:$H$8,MIN(C10,4))</f>
+        <v/>
+      </c>
+      <c r="M10" s="23">
+        <f>L10*C10*D10*H10</f>
+        <v/>
+      </c>
+      <c r="N10" s="23">
+        <f>M10-J10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>公式直販</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>二丁目</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="24">
+        <f>前提条件!$B$14</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>1-F11-G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="23">
+        <f>E11*C11*D11*H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="23">
+        <f>(IF(C11&lt;=3,前提条件!$B$6,IF(C11&lt;=6,前提条件!$B$7,前提条件!$B$8))+前提条件!$B$13)*D11</f>
+        <v/>
+      </c>
+      <c r="K11" s="23">
+        <f>I11-J11</f>
+        <v/>
+      </c>
+      <c r="L11" s="23">
+        <f>INDEX('公式価格（段階制）'!$B$5:$B$8,MIN(C11,4))</f>
+        <v/>
+      </c>
+      <c r="M11" s="23">
+        <f>L11*C11*D11*H11</f>
+        <v/>
+      </c>
+      <c r="N11" s="23">
+        <f>M11-J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C12" s="25">
+        <f>SUMPRODUCT(C5:C11,D5:D11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="25">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+      <c r="I12" s="26">
+        <f>SUM(I5:I11)</f>
+        <v/>
+      </c>
+      <c r="J12" s="26">
+        <f>SUM(J5:J11)</f>
+        <v/>
+      </c>
+      <c r="K12" s="26">
+        <f>SUM(K5:K11)</f>
+        <v/>
+      </c>
+      <c r="M12" s="26">
+        <f>SUM(M5:M11)</f>
+        <v/>
+      </c>
+      <c r="N12" s="26">
+        <f>SUM(N5:N11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>キャンセルで戻らなかったシステム利用料</t>
+        </is>
+      </c>
+      <c r="K13" s="23" t="n">
+        <v>-630</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>読み方</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>・利益の大半はKlook経由のハンコ（費用なし）。Reeluが案内するツアーは現行の一律価格だと1〜2名で赤字、段階制なら全人数で黒字。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>・新価格の列は需要が変わらない前提の試算。値上げで予約数が減る影響は含まない（推測）。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Pricing model: mark current prices as actuals, add update note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7xJuJLT164ew2d7KNvQh3
</commit_message>
<xml_diff>
--- a/docs/pricing/NGT_価格モデル.xlsx
+++ b/docs/pricing/NGT_価格モデル.xlsx
@@ -540,6 +540,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>最終更新：2026-10-02（手数料・システム利用料を LINKTIVITY 取引明細 2026/9 の実数に更新、ハンコの費用なしを反映、9月実績シートを追加）</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -768,7 +775,7 @@
           <t>現行 公式価格（1名あたり）</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="7" t="n">
         <v>2500</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -778,7 +785,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>サイト表示 $16.67 から推定（推測・要確認）</t>
+          <t>実数：LINKTIVITY取引明細（2026/9）の公式直販の単価</t>
         </is>
       </c>
     </row>
@@ -798,7 +805,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>「公式の方が500円安い」（ご本人回答）から算出</t>
+          <t>実数：LINKTIVITY取引明細（2026/9）。Klook・Travelers Road とも1名¥3,000</t>
         </is>
       </c>
     </row>
@@ -823,11 +830,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>チャネル別の手数料</t>
         </is>
       </c>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -2321,7 +2331,7 @@
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>・全件を公式価格で計算した試算（OTA経由分は手数料控除後の手取りがさらに低い）。ガイド費は特別単価を当てはめた仮定で、過去の実際のガイド費とは異なる。</t>
+          <t>・全件を公式価格（¥2,500）で計算した試算。OTA経由分は手取りがさらに低い（Klook 77%・Travelers Road 80%、公式直販 93%）。ガイド費は特別単価を当てはめた仮定で、過去の実際のガイド費とは異なる。ハンコツアー（費用なし）も同じガイド費で計算しているため、赤字回数は実際より多く出ている。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pricing model: use the current Reelu special rate as the basis; normal rate shown for reference
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7xJuJLT164ew2d7KNvQh3
</commit_message>
<xml_diff>
--- a/docs/pricing/NGT_価格モデル.xlsx
+++ b/docs/pricing/NGT_価格モデル.xlsx
@@ -642,7 +642,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>ガイド費（通常単価・7ヶ月目以降）</t>
+          <t>ガイド費（通常単価・7ヶ月目以降）【参考：計算の基準は特別単価】</t>
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
@@ -1044,7 +1044,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B5〜B8（青字）が提案価格。1名／2名／3名／4名以上の4段階で、4名以上は同額。</t>
+          <t>B5〜B8（青字）が提案価格。1名／2名／3名／4名以上の4段階で、4名以上は同額。利益の計算はReelu特別単価（現状の単価）が基準。通常単価の列は特別単価終了後の参考。</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>ガイド費（通常単価）</t>
+          <t>ガイド費（通常単価）【参考】</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>利益（通常単価）</t>
+          <t>利益（通常単価）【参考】</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>利益率（通常）</t>
+          <t>利益率（通常）【参考】</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>目標利益率に必要な1名単価（通常）</t>
+          <t>目標利益率に必要な1名単価（通常）【参考】</t>
         </is>
       </c>
     </row>

</xml_diff>